<commit_message>
Complete database-free extraction pipeline
</commit_message>
<xml_diff>
--- a/CIEH_Extraction/data/review/cieh_review.xlsx
+++ b/CIEH_Extraction/data/review/cieh_review.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Records" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Review Records'!$A$1:$P$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Review Records'!$A$1:$P$65</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -42,13 +42,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00244062"/>
-        <bgColor rgb="00244062"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -438,24 +436,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P87"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="65" customWidth="1" min="8" max="8"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
-    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -542,41 +540,47 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2016-17</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G2" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Year: 2016-17, Practitoner: 7</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2016-17, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J2" s="3" t="n"/>
@@ -588,41 +592,47 @@
       <c r="P2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>FOI002930_Response.pdf</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>FOI 443.xlsx</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>2016-17</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Year: 2016-17, Premises: 0</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2016-17, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J3" s="3" t="n"/>
@@ -634,41 +644,47 @@
       <c r="P3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>2017-18</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G4" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Year: 2017-18, Practitoner: 7</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2017-18, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J4" s="3" t="n"/>
@@ -680,41 +696,47 @@
       <c r="P4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2017-18</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G5" s="2" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Year: 2017-18, Premises: 0</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2017-18, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J5" s="3" t="n"/>
@@ -726,41 +748,47 @@
       <c r="P5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2018-19</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G6" s="2" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Year: 2018-19, Practitoner: 4</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2018-19, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J6" s="3" t="n"/>
@@ -772,41 +800,47 @@
       <c r="P6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="n"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2018-19</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G7" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Year: 2018-19, Premises: 1</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2018-19, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J7" s="3" t="n"/>
@@ -818,41 +852,47 @@
       <c r="P7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="n"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2019-20</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G8" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Year: 2019-20, Practitoner: 3</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2019-20, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J8" s="3" t="n"/>
@@ -864,41 +904,47 @@
       <c r="P8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2019-20</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Year: 2019-20, Premises: 0</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2019-20, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J9" s="3" t="n"/>
@@ -910,23 +956,29 @@
       <c r="P9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="n"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>2020-21</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>tattoo_premises</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -939,12 +991,12 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Year: 2020-21, Practitoner: 2</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2020-21, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J10" s="3" t="n"/>
@@ -956,41 +1008,47 @@
       <c r="P10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="n"/>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>2020-21</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G11" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Year: 2020-21, Premises: 1</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2020-21, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J11" s="3" t="n"/>
@@ -1002,41 +1060,47 @@
       <c r="P11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="2" t="n"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2021-22</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
+          <t>tattoo_premises</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G12" s="2" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Year: 2021-22, Practitoner: 8</t>
+          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2021-22, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J12" s="3" t="n"/>
@@ -1048,41 +1112,47 @@
       <c r="P12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="2" t="n"/>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2021-22</t>
+          <t>2015</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G13" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Year: 2021-22, Premises: 5</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2021-22, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J13" s="3" t="n"/>
@@ -1094,41 +1164,47 @@
       <c r="P13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="n"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2022-23</t>
+          <t>2016</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G14" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Year: 2022-23, Practitoner: 6</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2022-23, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J14" s="3" t="n"/>
@@ -1140,41 +1216,47 @@
       <c r="P14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="2" t="n"/>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>2022-23</t>
+          <t>2017</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G15" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Year: 2022-23, Premises: 1</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2022-23, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J15" s="3" t="n"/>
@@ -1186,41 +1268,47 @@
       <c r="P15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="2" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2023-24</t>
+          <t>2018</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G16" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Year: 2023-24, Practitoner: 11</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2023-24, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J16" s="3" t="n"/>
@@ -1232,41 +1320,47 @@
       <c r="P16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="2" t="n"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>2023-24</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G17" s="2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Year: 2023-24, Premises: 6</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2023-24, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J17" s="3" t="n"/>
@@ -1278,41 +1372,47 @@
       <c r="P17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="2" t="n"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2024-25</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G18" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Year: 2024-25, Practitoner: 3</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2024-25, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J18" s="3" t="n"/>
@@ -1324,41 +1424,47 @@
       <c r="P18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="n"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>2024-25</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G19" s="2" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Year: 2024-25, Premises: 2</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2024-25, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J19" s="3" t="n"/>
@@ -1370,41 +1476,47 @@
       <c r="P19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G20" s="2" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Year: 2025-26, Practitoner: 7</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2025-26, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J20" s="3" t="n"/>
@@ -1416,41 +1528,47 @@
       <c r="P20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="n"/>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>2025-26</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G21" s="2" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Year: 2025-26, Premises: 4</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2025-26, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J21" s="3" t="n"/>
@@ -1462,41 +1580,47 @@
       <c r="P21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>2026-27</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G22" s="2" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Year: 2026-27, Practitoner: 5</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2026-27, Practitoner column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J22" s="3" t="n"/>
@@ -1508,41 +1632,47 @@
       <c r="P22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>50bd7a00375cbe659481011f67cd3b138c5ef84473c1914e0eb3c764acf0431b-0022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+        </is>
+      </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>FOI 443.xlsx</t>
+          <t>FOI002930_Response.pdf</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-27</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
+          <t>tattoo_practitioners</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
       <c r="G23" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Year: 2026-27, Premises: 2</t>
+          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Sheet '10 Years', row 2026-27, Premises column</t>
+          <t>Our Response, Q2</t>
         </is>
       </c>
       <c r="J23" s="3" t="n"/>
@@ -1554,8 +1684,10 @@
       <c r="P23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0001</t>
+        </is>
       </c>
       <c r="B24" s="2" t="n"/>
       <c r="C24" s="2" t="inlineStr">
@@ -1600,8 +1732,10 @@
       <c r="P24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>24</v>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0002</t>
+        </is>
       </c>
       <c r="B25" s="2" t="n"/>
       <c r="C25" s="2" t="inlineStr">
@@ -1646,8 +1780,10 @@
       <c r="P25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0003</t>
+        </is>
       </c>
       <c r="B26" s="2" t="n"/>
       <c r="C26" s="2" t="inlineStr">
@@ -1692,8 +1828,10 @@
       <c r="P26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>26</v>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0004</t>
+        </is>
       </c>
       <c r="B27" s="2" t="n"/>
       <c r="C27" s="2" t="inlineStr">
@@ -1738,8 +1876,10 @@
       <c r="P27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>27</v>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0005</t>
+        </is>
       </c>
       <c r="B28" s="2" t="n"/>
       <c r="C28" s="2" t="inlineStr">
@@ -1784,8 +1924,10 @@
       <c r="P28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>28</v>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0006</t>
+        </is>
       </c>
       <c r="B29" s="2" t="n"/>
       <c r="C29" s="2" t="inlineStr">
@@ -1830,8 +1972,10 @@
       <c r="P29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>29</v>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0007</t>
+        </is>
       </c>
       <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="inlineStr">
@@ -1876,8 +2020,10 @@
       <c r="P30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>30</v>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0008</t>
+        </is>
       </c>
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="inlineStr">
@@ -1922,8 +2068,10 @@
       <c r="P31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>31</v>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0009</t>
+        </is>
       </c>
       <c r="B32" s="2" t="n"/>
       <c r="C32" s="2" t="inlineStr">
@@ -1968,8 +2116,10 @@
       <c r="P32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>32</v>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0010</t>
+        </is>
       </c>
       <c r="B33" s="2" t="n"/>
       <c r="C33" s="2" t="inlineStr">
@@ -2014,8 +2164,10 @@
       <c r="P33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0011</t>
+        </is>
       </c>
       <c r="B34" s="2" t="n"/>
       <c r="C34" s="2" t="inlineStr">
@@ -2060,8 +2212,10 @@
       <c r="P34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>34</v>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0012</t>
+        </is>
       </c>
       <c r="B35" s="2" t="n"/>
       <c r="C35" s="2" t="inlineStr">
@@ -2106,8 +2260,10 @@
       <c r="P35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0013</t>
+        </is>
       </c>
       <c r="B36" s="2" t="n"/>
       <c r="C36" s="2" t="inlineStr">
@@ -2152,8 +2308,10 @@
       <c r="P36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>36</v>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0014</t>
+        </is>
       </c>
       <c r="B37" s="2" t="n"/>
       <c r="C37" s="2" t="inlineStr">
@@ -2198,8 +2356,10 @@
       <c r="P37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0015</t>
+        </is>
       </c>
       <c r="B38" s="2" t="n"/>
       <c r="C38" s="2" t="inlineStr">
@@ -2244,8 +2404,10 @@
       <c r="P38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0016</t>
+        </is>
       </c>
       <c r="B39" s="2" t="n"/>
       <c r="C39" s="2" t="inlineStr">
@@ -2290,8 +2452,10 @@
       <c r="P39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0017</t>
+        </is>
       </c>
       <c r="B40" s="2" t="n"/>
       <c r="C40" s="2" t="inlineStr">
@@ -2336,8 +2500,10 @@
       <c r="P40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0018</t>
+        </is>
       </c>
       <c r="B41" s="2" t="n"/>
       <c r="C41" s="2" t="inlineStr">
@@ -2382,8 +2548,10 @@
       <c r="P41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0019</t>
+        </is>
       </c>
       <c r="B42" s="2" t="n"/>
       <c r="C42" s="2" t="inlineStr">
@@ -2428,8 +2596,10 @@
       <c r="P42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>42</v>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0020</t>
+        </is>
       </c>
       <c r="B43" s="2" t="n"/>
       <c r="C43" s="2" t="inlineStr">
@@ -2474,8 +2644,10 @@
       <c r="P43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>43</v>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0021</t>
+        </is>
       </c>
       <c r="B44" s="2" t="n"/>
       <c r="C44" s="2" t="inlineStr">
@@ -2520,8 +2692,10 @@
       <c r="P44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>44</v>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>98e80d95caaba97d57e26a4a5ba5a5c1f41a5e91b0f616240ae0857218e75e61-0022</t>
+        </is>
       </c>
       <c r="B45" s="2" t="n"/>
       <c r="C45" s="2" t="inlineStr">
@@ -2566,22 +2740,24 @@
       <c r="P45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>45</v>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0001</t>
+        </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2591,20 +2767,20 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>Q2) Please advise, based on your Environmental Health or Licensing records, how many premises that specialised in the provision of tattooing services or tattoo studios were licensed (special treatment premises) with you during each financial year... Financial Year: 2016/17 Number of Licensed Tattoo Premises: 15</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 1</t>
         </is>
       </c>
       <c r="J46" s="3" t="n"/>
@@ -2616,22 +2792,24 @@
       <c r="P46" s="3" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>46</v>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0002</t>
+        </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2017/18</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2641,20 +2819,20 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G47" s="2" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2017/18 16</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 2</t>
         </is>
       </c>
       <c r="J47" s="3" t="n"/>
@@ -2666,22 +2844,24 @@
       <c r="P47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0003</t>
+        </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2691,20 +2871,20 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2018/19 14</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 3</t>
         </is>
       </c>
       <c r="J48" s="3" t="n"/>
@@ -2716,22 +2896,24 @@
       <c r="P48" s="3" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>48</v>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0004</t>
+        </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -2741,20 +2923,20 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2019/20 16</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 4</t>
         </is>
       </c>
       <c r="J49" s="3" t="n"/>
@@ -2766,22 +2948,24 @@
       <c r="P49" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>49</v>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0005</t>
+        </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2791,20 +2975,20 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G50" s="2" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2020/21 16</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 5</t>
         </is>
       </c>
       <c r="J50" s="3" t="n"/>
@@ -2816,22 +3000,24 @@
       <c r="P50" s="3" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>50</v>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0006</t>
+        </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -2841,20 +3027,20 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G51" s="2" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2021/22 17</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 6</t>
         </is>
       </c>
       <c r="J51" s="3" t="n"/>
@@ -2866,22 +3052,24 @@
       <c r="P51" s="3" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>51</v>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0007</t>
+        </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2891,20 +3079,20 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G52" s="2" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2022/23 18</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 7</t>
         </is>
       </c>
       <c r="J52" s="3" t="n"/>
@@ -2916,22 +3104,24 @@
       <c r="P52" s="3" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>52</v>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0008</t>
+        </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2023/24</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -2941,20 +3131,20 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G53" s="2" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2023/24 20</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 8</t>
         </is>
       </c>
       <c r="J53" s="3" t="n"/>
@@ -2966,22 +3156,24 @@
       <c r="P53" s="3" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>53</v>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0009</t>
+        </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2991,20 +3183,20 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G54" s="2" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2024/25 23</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 9</t>
         </is>
       </c>
       <c r="J54" s="3" t="n"/>
@@ -3016,22 +3208,24 @@
       <c r="P54" s="3" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n">
-        <v>54</v>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0010</t>
+        </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3041,20 +3235,20 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G55" s="2" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>2025/26 21</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2 table, row 10</t>
         </is>
       </c>
       <c r="J55" s="3" t="n"/>
@@ -3066,45 +3260,47 @@
       <c r="P55" s="3" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>55</v>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0011</t>
+        </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2016/17</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>tattoo_premises</t>
+          <t>tattoo_practitioners</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G56" s="2" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Premises 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 3 9 2 13 6 5 11 7 4 2 3</t>
+          <t>Q2a) and how many individual practitioners within the aforementioned premises were licensed, or covered by a license, in total during each financial year... Financial Year: 2016/17 Total Practitioners: 28</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 1</t>
         </is>
       </c>
       <c r="J56" s="3" t="n"/>
@@ -3116,22 +3312,24 @@
       <c r="P56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n">
-        <v>56</v>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0012</t>
+        </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>2015</t>
+          <t>2017/18</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3141,20 +3339,20 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G57" s="2" t="n">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2017/18 27</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 2</t>
         </is>
       </c>
       <c r="J57" s="3" t="n"/>
@@ -3166,22 +3364,24 @@
       <c r="P57" s="3" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n">
-        <v>57</v>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0013</t>
+        </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>2016</t>
+          <t>2018/19</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3191,20 +3391,20 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G58" s="2" t="n">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2018/19 28</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 3</t>
         </is>
       </c>
       <c r="J58" s="3" t="n"/>
@@ -3216,22 +3416,24 @@
       <c r="P58" s="3" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>58</v>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0014</t>
+        </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>2017</t>
+          <t>2019/20</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -3241,20 +3443,20 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G59" s="2" t="n">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2019/20 31</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 4</t>
         </is>
       </c>
       <c r="J59" s="3" t="n"/>
@@ -3266,22 +3468,24 @@
       <c r="P59" s="3" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n">
-        <v>59</v>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0015</t>
+        </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>2020/21</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3291,20 +3495,20 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G60" s="2" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2020/21 33</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 5</t>
         </is>
       </c>
       <c r="J60" s="3" t="n"/>
@@ -3316,22 +3520,24 @@
       <c r="P60" s="3" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n">
-        <v>60</v>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0016</t>
+        </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2021/22</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3341,20 +3547,20 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G61" s="2" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2021/22 34</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 6</t>
         </is>
       </c>
       <c r="J61" s="3" t="n"/>
@@ -3366,22 +3572,24 @@
       <c r="P61" s="3" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n">
-        <v>61</v>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0017</t>
+        </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2022/23</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3391,20 +3599,20 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G62" s="2" t="n">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2022/23 60</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 7</t>
         </is>
       </c>
       <c r="J62" s="3" t="n"/>
@@ -3416,22 +3624,24 @@
       <c r="P62" s="3" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n">
-        <v>62</v>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0018</t>
+        </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2023/24</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -3441,20 +3651,20 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G63" s="2" t="n">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2023/24 68</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 8</t>
         </is>
       </c>
       <c r="J63" s="3" t="n"/>
@@ -3466,22 +3676,24 @@
       <c r="P63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n">
-        <v>63</v>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0019</t>
+        </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024/25</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3491,20 +3703,20 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2024/25 82</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 9</t>
         </is>
       </c>
       <c r="J64" s="3" t="n"/>
@@ -3516,22 +3728,24 @@
       <c r="P64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n">
-        <v>64</v>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>ee25eb85eef9fa11cfd1d2f40df3f748fb3963a6f145310c2c164be1ad5966e0-0020</t>
+        </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
+          <t>London Borough of Lewisham</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>FOI002930_Response.pdf</t>
+          <t>Lewisham_Borough_Council.txt</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2025/26</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -3541,20 +3755,20 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>active_register_total</t>
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>11</v>
+        <v>79</v>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
+          <t>2025/26 79</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Our Response, Q2</t>
+          <t>Q2a table, row 10</t>
         </is>
       </c>
       <c r="J65" s="3" t="n"/>
@@ -3565,1110 +3779,10 @@
       <c r="O65" s="3" t="n"/>
       <c r="P65" s="3" t="n"/>
     </row>
-    <row r="66">
-      <c r="A66" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>FOI002930_Response.pdf</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>Our Response, Q2</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="n"/>
-      <c r="K66" s="3" t="n"/>
-      <c r="L66" s="3" t="n"/>
-      <c r="M66" s="3" t="n"/>
-      <c r="N66" s="3" t="n"/>
-      <c r="O66" s="3" t="n"/>
-      <c r="P66" s="3" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Royal Borough of Windsor &amp; Maidenhead</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>FOI002930_Response.pdf</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="H67" s="2" t="inlineStr">
-        <is>
-          <t>Practitioners 2025 2024 2023 2022 2021 2020 2019 2018 2017 2016 2015 6 14 11 14 11 7 14 16 7 2 4</t>
-        </is>
-      </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>Our Response, Q2</t>
-        </is>
-      </c>
-      <c r="J67" s="3" t="n"/>
-      <c r="K67" s="3" t="n"/>
-      <c r="L67" s="3" t="n"/>
-      <c r="M67" s="3" t="n"/>
-      <c r="N67" s="3" t="n"/>
-      <c r="O67" s="3" t="n"/>
-      <c r="P67" s="3" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>2016/17</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="H68" s="2" t="inlineStr">
-        <is>
-          <t>Q2) Please advise, based on your Environmental Health or Licensing records, how many premises that specialised in the provision of tattooing services or tattoo studios were licensed (special treatment premises) with you during each financial year... Financial Year: 2016/17 Number of Licensed Tattoo Premises: 15</t>
-        </is>
-      </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 1</t>
-        </is>
-      </c>
-      <c r="J68" s="3" t="n"/>
-      <c r="K68" s="3" t="n"/>
-      <c r="L68" s="3" t="n"/>
-      <c r="M68" s="3" t="n"/>
-      <c r="N68" s="3" t="n"/>
-      <c r="O68" s="3" t="n"/>
-      <c r="P68" s="3" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>2017/18</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>2017/18 16</t>
-        </is>
-      </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 2</t>
-        </is>
-      </c>
-      <c r="J69" s="3" t="n"/>
-      <c r="K69" s="3" t="n"/>
-      <c r="L69" s="3" t="n"/>
-      <c r="M69" s="3" t="n"/>
-      <c r="N69" s="3" t="n"/>
-      <c r="O69" s="3" t="n"/>
-      <c r="P69" s="3" t="n"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>2018/19</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="H70" s="2" t="inlineStr">
-        <is>
-          <t>2018/19 14</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 3</t>
-        </is>
-      </c>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="3" t="n"/>
-      <c r="L70" s="3" t="n"/>
-      <c r="M70" s="3" t="n"/>
-      <c r="N70" s="3" t="n"/>
-      <c r="O70" s="3" t="n"/>
-      <c r="P70" s="3" t="n"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>2019/20</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>2019/20 16</t>
-        </is>
-      </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 4</t>
-        </is>
-      </c>
-      <c r="J71" s="3" t="n"/>
-      <c r="K71" s="3" t="n"/>
-      <c r="L71" s="3" t="n"/>
-      <c r="M71" s="3" t="n"/>
-      <c r="N71" s="3" t="n"/>
-      <c r="O71" s="3" t="n"/>
-      <c r="P71" s="3" t="n"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>2020/21</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="n">
-        <v>16</v>
-      </c>
-      <c r="H72" s="2" t="inlineStr">
-        <is>
-          <t>2020/21 16</t>
-        </is>
-      </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 5</t>
-        </is>
-      </c>
-      <c r="J72" s="3" t="n"/>
-      <c r="K72" s="3" t="n"/>
-      <c r="L72" s="3" t="n"/>
-      <c r="M72" s="3" t="n"/>
-      <c r="N72" s="3" t="n"/>
-      <c r="O72" s="3" t="n"/>
-      <c r="P72" s="3" t="n"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>2021/22</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="H73" s="2" t="inlineStr">
-        <is>
-          <t>2021/22 17</t>
-        </is>
-      </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 6</t>
-        </is>
-      </c>
-      <c r="J73" s="3" t="n"/>
-      <c r="K73" s="3" t="n"/>
-      <c r="L73" s="3" t="n"/>
-      <c r="M73" s="3" t="n"/>
-      <c r="N73" s="3" t="n"/>
-      <c r="O73" s="3" t="n"/>
-      <c r="P73" s="3" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>2022/23</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>2022/23 18</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 7</t>
-        </is>
-      </c>
-      <c r="J74" s="3" t="n"/>
-      <c r="K74" s="3" t="n"/>
-      <c r="L74" s="3" t="n"/>
-      <c r="M74" s="3" t="n"/>
-      <c r="N74" s="3" t="n"/>
-      <c r="O74" s="3" t="n"/>
-      <c r="P74" s="3" t="n"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>2023/24</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>2023/24 20</t>
-        </is>
-      </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 8</t>
-        </is>
-      </c>
-      <c r="J75" s="3" t="n"/>
-      <c r="K75" s="3" t="n"/>
-      <c r="L75" s="3" t="n"/>
-      <c r="M75" s="3" t="n"/>
-      <c r="N75" s="3" t="n"/>
-      <c r="O75" s="3" t="n"/>
-      <c r="P75" s="3" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>2024/25</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>2024/25 23</t>
-        </is>
-      </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 9</t>
-        </is>
-      </c>
-      <c r="J76" s="3" t="n"/>
-      <c r="K76" s="3" t="n"/>
-      <c r="L76" s="3" t="n"/>
-      <c r="M76" s="3" t="n"/>
-      <c r="N76" s="3" t="n"/>
-      <c r="O76" s="3" t="n"/>
-      <c r="P76" s="3" t="n"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="n">
-        <v>76</v>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>2025/26</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_premises</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="H77" s="2" t="inlineStr">
-        <is>
-          <t>2025/26 21</t>
-        </is>
-      </c>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>Q2 table, row 10</t>
-        </is>
-      </c>
-      <c r="J77" s="3" t="n"/>
-      <c r="K77" s="3" t="n"/>
-      <c r="L77" s="3" t="n"/>
-      <c r="M77" s="3" t="n"/>
-      <c r="N77" s="3" t="n"/>
-      <c r="O77" s="3" t="n"/>
-      <c r="P77" s="3" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>2016/17</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>Q2a) and how many individual practitioners within the aforementioned premises were licensed, or covered by a license, in total during each financial year... Financial Year: 2016/17 Total Practitioners: 28</t>
-        </is>
-      </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 1</t>
-        </is>
-      </c>
-      <c r="J78" s="3" t="n"/>
-      <c r="K78" s="3" t="n"/>
-      <c r="L78" s="3" t="n"/>
-      <c r="M78" s="3" t="n"/>
-      <c r="N78" s="3" t="n"/>
-      <c r="O78" s="3" t="n"/>
-      <c r="P78" s="3" t="n"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>2017/18</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="H79" s="2" t="inlineStr">
-        <is>
-          <t>2017/18 27</t>
-        </is>
-      </c>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 2</t>
-        </is>
-      </c>
-      <c r="J79" s="3" t="n"/>
-      <c r="K79" s="3" t="n"/>
-      <c r="L79" s="3" t="n"/>
-      <c r="M79" s="3" t="n"/>
-      <c r="N79" s="3" t="n"/>
-      <c r="O79" s="3" t="n"/>
-      <c r="P79" s="3" t="n"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>2018/19</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>2018/19 28</t>
-        </is>
-      </c>
-      <c r="I80" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 3</t>
-        </is>
-      </c>
-      <c r="J80" s="3" t="n"/>
-      <c r="K80" s="3" t="n"/>
-      <c r="L80" s="3" t="n"/>
-      <c r="M80" s="3" t="n"/>
-      <c r="N80" s="3" t="n"/>
-      <c r="O80" s="3" t="n"/>
-      <c r="P80" s="3" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>2019/20</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G81" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
-        <is>
-          <t>2019/20 31</t>
-        </is>
-      </c>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 4</t>
-        </is>
-      </c>
-      <c r="J81" s="3" t="n"/>
-      <c r="K81" s="3" t="n"/>
-      <c r="L81" s="3" t="n"/>
-      <c r="M81" s="3" t="n"/>
-      <c r="N81" s="3" t="n"/>
-      <c r="O81" s="3" t="n"/>
-      <c r="P81" s="3" t="n"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>2020/21</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
-        <is>
-          <t>2020/21 33</t>
-        </is>
-      </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 5</t>
-        </is>
-      </c>
-      <c r="J82" s="3" t="n"/>
-      <c r="K82" s="3" t="n"/>
-      <c r="L82" s="3" t="n"/>
-      <c r="M82" s="3" t="n"/>
-      <c r="N82" s="3" t="n"/>
-      <c r="O82" s="3" t="n"/>
-      <c r="P82" s="3" t="n"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>2021/22</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
-        <is>
-          <t>2021/22 34</t>
-        </is>
-      </c>
-      <c r="I83" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 6</t>
-        </is>
-      </c>
-      <c r="J83" s="3" t="n"/>
-      <c r="K83" s="3" t="n"/>
-      <c r="L83" s="3" t="n"/>
-      <c r="M83" s="3" t="n"/>
-      <c r="N83" s="3" t="n"/>
-      <c r="O83" s="3" t="n"/>
-      <c r="P83" s="3" t="n"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>2022/23</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>2022/23 60</t>
-        </is>
-      </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 7</t>
-        </is>
-      </c>
-      <c r="J84" s="3" t="n"/>
-      <c r="K84" s="3" t="n"/>
-      <c r="L84" s="3" t="n"/>
-      <c r="M84" s="3" t="n"/>
-      <c r="N84" s="3" t="n"/>
-      <c r="O84" s="3" t="n"/>
-      <c r="P84" s="3" t="n"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>2023/24</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G85" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>2023/24 68</t>
-        </is>
-      </c>
-      <c r="I85" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 8</t>
-        </is>
-      </c>
-      <c r="J85" s="3" t="n"/>
-      <c r="K85" s="3" t="n"/>
-      <c r="L85" s="3" t="n"/>
-      <c r="M85" s="3" t="n"/>
-      <c r="N85" s="3" t="n"/>
-      <c r="O85" s="3" t="n"/>
-      <c r="P85" s="3" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>2024/25</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G86" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H86" s="2" t="inlineStr">
-        <is>
-          <t>2024/25 82</t>
-        </is>
-      </c>
-      <c r="I86" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 9</t>
-        </is>
-      </c>
-      <c r="J86" s="3" t="n"/>
-      <c r="K86" s="3" t="n"/>
-      <c r="L86" s="3" t="n"/>
-      <c r="M86" s="3" t="n"/>
-      <c r="N86" s="3" t="n"/>
-      <c r="O86" s="3" t="n"/>
-      <c r="P86" s="3" t="n"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>London Borough of Lewisham</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>Lewisham_Borough_Council.txt</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>2025/26</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>tattoo_practitioners</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>active_register_total</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
-        <is>
-          <t>2025/26 79</t>
-        </is>
-      </c>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t>Q2a table, row 10</t>
-        </is>
-      </c>
-      <c r="J87" s="3" t="n"/>
-      <c r="K87" s="3" t="n"/>
-      <c r="L87" s="3" t="n"/>
-      <c r="M87" s="3" t="n"/>
-      <c r="N87" s="3" t="n"/>
-      <c r="O87" s="3" t="n"/>
-      <c r="P87" s="3" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:P87"/>
+  <autoFilter ref="A1:P65"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J65" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"approved,rejected,corrected"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>